<commit_message>
Recompute breakout screener across all 173 F&O tickers
Adds run_consolidated_screener.py, which reads every per-ticker
historical JSON file under data/nse_historical/2026-08-15/ (25 tickers
from the initial run plus 148 fetched across 5 batches) and reapplies
the original DMA/CAR breakout screen in one consistent pass, replacing
the earlier partial (25-ticker) Breakout_Stocks output.

Result: 173/173 tickers resolved and screened, 0 skipped, 0 stocks
met all 5 breakout criteria today.
</commit_message>
<xml_diff>
--- a/data/nse_historical/2026-08-15/screener/Breakout_Stocks_2026-08-15.xlsx
+++ b/data/nse_historical/2026-08-15/screener/Breakout_Stocks_2026-08-15.xlsx
@@ -413,47 +413,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Current Price</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>30 DMA</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>50 DMA</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>200 DMA</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Distance to 200 DMA (%)</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>CAR (10 Days)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>